<commit_message>
fix(review): pass-through parts screen rename cleanup
- Finding 1: rewrite FAT-INSP-040 (docs/fat/areas/inspection.csv) for the
  Inventory/Assembly tab shell, adding the only witnessable check of the
  cross-tab inventoryChanged broadcast; relabel the FAT sheet in
  build_fat_workbook.js and regenerate the committed MPP_MES_FAT.xlsx
- Finding 2: sync the DefaultScreen dropdown label in
  BlueRidge/Location/AttributeOptions/code.py with the page-config title
  "Pass-Through Parts" (route string unchanged)
- Finding 3: drop the inaccurate "(FIFO by arrival)" claim from the
  ReceivingDock on-hand panel header - the consume path orders by
  CreatedAt, not arrival-into-cell time
- Finding 4: correct design spec S6.3, which stated the fallback-terminal
  risk backwards; Lot_Create and Assembly_CompleteTray both fail closed
  with an operator-visible eligibility message because
  ufn_AncestorLocationIds only walks upward, so a whole-site zone's
  ancestor set contains no configured cell
</commit_message>
<xml_diff>
--- a/docs/fat/MPP_MES_FAT.xlsx
+++ b/docs/fat/MPP_MES_FAT.xlsx
@@ -21,7 +21,7 @@
     <sheet sheetId="14" name="Trim" state="visible" r:id="rId18"/>
     <sheet sheetId="15" name="Machining" state="visible" r:id="rId19"/>
     <sheet sheetId="16" name="Assembly" state="visible" r:id="rId20"/>
-    <sheet sheetId="17" name="Third-Party Inspection" state="visible" r:id="rId21"/>
+    <sheet sheetId="17" name="Pass-Through Parts" state="visible" r:id="rId21"/>
     <sheet sheetId="18" name="Quality Capture &amp; Holds" state="visible" r:id="rId22"/>
     <sheet sheetId="19" name="Movements &amp; Inventory" state="visible" r:id="rId23"/>
     <sheet sheetId="20" name="LOT Traceability &amp; Genealogy" state="visible" r:id="rId24"/>
@@ -180,7 +180,7 @@
     <t>Assembly</t>
   </si>
   <si>
-    <t>Third-Party Inspection</t>
+    <t>Pass-Through Parts</t>
   </si>
   <si>
     <t>Quality Capture &amp; Holds</t>
@@ -6405,19 +6405,19 @@
     <t>FAT-INSP-040</t>
   </si>
   <si>
-    <t>Third-party inspection check-in</t>
-  </si>
-  <si>
-    <t>A third-party inspection terminal</t>
-  </si>
-  <si>
-    <t>Use the Check In tab to receive a vendor LOT into the inspection queue</t>
-  </si>
-  <si>
-    <t>The Check In tab (embedded Receiving Dock) creates the received LOT and it appears in the Inspect-tab queue for the station</t>
-  </si>
-  <si>
-    <t>BRA — third-party inspection station wiring</t>
+    <t>Pass-through parts receive</t>
+  </si>
+  <si>
+    <t>A pass-through parts terminal</t>
+  </si>
+  <si>
+    <t>Use the Inventory tab to receive a vendor LOT</t>
+  </si>
+  <si>
+    <t>The Inventory tab (embedded Receiving Dock) creates the received LOT, prints its LTT, and the LOT appears in the Inventory tab's on-hand panel AND in the Assembly tab's component projection without pressing Refresh</t>
+  </si>
+  <si>
+    <t>BRA — pass-through parts station wiring (cross-tab inventoryChanged broadcast)</t>
   </si>
   <si>
     <t>FDS-05-013  —  Status Codes      (FRS 3.16.3)</t>
@@ -21189,7 +21189,7 @@
       <c r="H7" s="29"/>
       <c r="I7" s="29"/>
     </row>
-    <row r="8" ht="41.8" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" ht="79.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
         <v>2122</v>
       </c>
@@ -29125,13 +29125,13 @@
         <v>4</v>
       </c>
       <c r="C39" s="12">
-        <f>COUNTIF('Third-Party Inspection'!F:F,"Pass")</f>
+        <f>COUNTIF('Pass-Through Parts'!F:F,"Pass")</f>
       </c>
       <c r="D39" s="12">
-        <f>COUNTIF('Third-Party Inspection'!F:F,"Fail")</f>
+        <f>COUNTIF('Pass-Through Parts'!F:F,"Fail")</f>
       </c>
       <c r="E39" s="12">
-        <f>COUNTIF('Third-Party Inspection'!F:F,"N/A")</f>
+        <f>COUNTIF('Pass-Through Parts'!F:F,"N/A")</f>
       </c>
       <c r="F39" s="12">
         <f>B39-C39-D39-E39</f>

</xml_diff>